<commit_message>
data up to 07/2025
</commit_message>
<xml_diff>
--- a/Data cleansing/output data/Просуммированные по категориям.xlsx
+++ b/Data cleansing/output data/Просуммированные по категориям.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DR169"/>
+  <dimension ref="A1:DY169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1039,6 +1039,41 @@
           <t>2024-12</t>
         </is>
       </c>
+      <c r="DS1" s="1" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="DT1" s="1" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="DU1" s="1" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="DV1" s="1" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="DW1" s="1" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="DX1" s="1" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="DY1" s="1" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1411,6 +1446,27 @@
       <c r="DR2" t="n">
         <v>0</v>
       </c>
+      <c r="DS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1783,6 +1839,27 @@
       <c r="DR3" t="n">
         <v>538.4</v>
       </c>
+      <c r="DS3" t="n">
+        <v>129.3</v>
+      </c>
+      <c r="DT3" t="n">
+        <v>77.59999999999999</v>
+      </c>
+      <c r="DU3" t="n">
+        <v>411.5</v>
+      </c>
+      <c r="DV3" t="n">
+        <v>128.1</v>
+      </c>
+      <c r="DW3" t="n">
+        <v>235.7</v>
+      </c>
+      <c r="DX3" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="DY3" t="n">
+        <v>25.17</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2155,6 +2232,27 @@
       <c r="DR4" t="n">
         <v>12.6</v>
       </c>
+      <c r="DS4" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="DT4" t="n">
+        <v>19</v>
+      </c>
+      <c r="DU4" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="DV4" t="n">
+        <v>12</v>
+      </c>
+      <c r="DW4" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="DX4" t="n">
+        <v>41.59999999999999</v>
+      </c>
+      <c r="DY4" t="n">
+        <v>28.1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2527,6 +2625,27 @@
       <c r="DR5" t="n">
         <v>930.28</v>
       </c>
+      <c r="DS5" t="n">
+        <v>322.1</v>
+      </c>
+      <c r="DT5" t="n">
+        <v>286.54</v>
+      </c>
+      <c r="DU5" t="n">
+        <v>447.4</v>
+      </c>
+      <c r="DV5" t="n">
+        <v>266.8</v>
+      </c>
+      <c r="DW5" t="n">
+        <v>496.55</v>
+      </c>
+      <c r="DX5" t="n">
+        <v>688</v>
+      </c>
+      <c r="DY5" t="n">
+        <v>212.7</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2899,6 +3018,27 @@
       <c r="DR6" t="n">
         <v>0</v>
       </c>
+      <c r="DS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT6" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="DU6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV6" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="DW6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="DX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY6" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3271,6 +3411,27 @@
       <c r="DR7" t="n">
         <v>0</v>
       </c>
+      <c r="DS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3641,6 +3802,27 @@
         <v>0</v>
       </c>
       <c r="DR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3933,6 +4115,27 @@
       <c r="DR9" t="n">
         <v>0</v>
       </c>
+      <c r="DS9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4305,6 +4508,27 @@
       <c r="DR10" t="n">
         <v>5.8</v>
       </c>
+      <c r="DS10" t="n">
+        <v>109.8</v>
+      </c>
+      <c r="DT10" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="DU10" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="DV10" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="DW10" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="DX10" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="DY10" t="n">
+        <v>14.2</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4677,6 +4901,27 @@
       <c r="DR11" t="n">
         <v>18.4</v>
       </c>
+      <c r="DS11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="DT11" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="DU11" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="DV11" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="DW11" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="DX11" t="n">
+        <v>59.92</v>
+      </c>
+      <c r="DY11" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5049,6 +5294,27 @@
       <c r="DR12" t="n">
         <v>0</v>
       </c>
+      <c r="DS12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="DT12" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU12" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="DV12" t="n">
+        <v>2</v>
+      </c>
+      <c r="DW12" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="DX12" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="DY12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5421,6 +5687,27 @@
       <c r="DR13" t="n">
         <v>1.2</v>
       </c>
+      <c r="DS13" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT13" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU13" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV13" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW13" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX13" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5793,6 +6080,27 @@
       <c r="DR14" t="n">
         <v>1740.77</v>
       </c>
+      <c r="DS14" t="n">
+        <v>450.07</v>
+      </c>
+      <c r="DT14" t="n">
+        <v>376.72</v>
+      </c>
+      <c r="DU14" t="n">
+        <v>335.32</v>
+      </c>
+      <c r="DV14" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="DW14" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="DX14" t="n">
+        <v>56.94</v>
+      </c>
+      <c r="DY14" t="n">
+        <v>13.58</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6164,6 +6472,27 @@
       </c>
       <c r="DR15" t="n">
         <v>921.4000000000001</v>
+      </c>
+      <c r="DS15" t="n">
+        <v>164</v>
+      </c>
+      <c r="DT15" t="n">
+        <v>580.5</v>
+      </c>
+      <c r="DU15" t="n">
+        <v>109.58</v>
+      </c>
+      <c r="DV15" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="DW15" t="n">
+        <v>174.45</v>
+      </c>
+      <c r="DX15" t="n">
+        <v>317.85</v>
+      </c>
+      <c r="DY15" t="n">
+        <v>163.8</v>
       </c>
     </row>
     <row r="16">
@@ -6359,6 +6688,27 @@
       <c r="DR16" t="n">
         <v>17.1</v>
       </c>
+      <c r="DS16" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="DT16" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="DU16" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV16" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="DW16" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX16" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="DY16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6553,6 +6903,27 @@
       <c r="DR17" t="n">
         <v>1.9</v>
       </c>
+      <c r="DS17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="DU17" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="DV17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX17" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="DY17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6747,6 +7118,27 @@
       <c r="DR18" t="n">
         <v>0</v>
       </c>
+      <c r="DS18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX18" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7119,6 +7511,27 @@
       <c r="DR19" t="n">
         <v>0</v>
       </c>
+      <c r="DS19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX19" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7491,6 +7904,27 @@
       <c r="DR20" t="n">
         <v>4952.389999999999</v>
       </c>
+      <c r="DS20" t="n">
+        <v>1275.12</v>
+      </c>
+      <c r="DT20" t="n">
+        <v>1448.13</v>
+      </c>
+      <c r="DU20" t="n">
+        <v>1486.2</v>
+      </c>
+      <c r="DV20" t="n">
+        <v>684.65</v>
+      </c>
+      <c r="DW20" t="n">
+        <v>1078.02</v>
+      </c>
+      <c r="DX20" t="n">
+        <v>1340.09</v>
+      </c>
+      <c r="DY20" t="n">
+        <v>503.05</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7861,6 +8295,27 @@
         <v>0</v>
       </c>
       <c r="DR21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX21" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8153,6 +8608,27 @@
       <c r="DR22" t="n">
         <v>764.4399999999999</v>
       </c>
+      <c r="DS22" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="DT22" t="n">
+        <v>60.13</v>
+      </c>
+      <c r="DU22" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="DV22" t="n">
+        <v>85.80000000000001</v>
+      </c>
+      <c r="DW22" t="n">
+        <v>96.61000000000001</v>
+      </c>
+      <c r="DX22" t="n">
+        <v>105</v>
+      </c>
+      <c r="DY22" t="n">
+        <v>44.09999999999999</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8525,6 +9001,27 @@
       <c r="DR23" t="n">
         <v>4253.58</v>
       </c>
+      <c r="DS23" t="n">
+        <v>3947.99</v>
+      </c>
+      <c r="DT23" t="n">
+        <v>3588.93</v>
+      </c>
+      <c r="DU23" t="n">
+        <v>4315.53</v>
+      </c>
+      <c r="DV23" t="n">
+        <v>3934.11</v>
+      </c>
+      <c r="DW23" t="n">
+        <v>3766.97</v>
+      </c>
+      <c r="DX23" t="n">
+        <v>4346.53</v>
+      </c>
+      <c r="DY23" t="n">
+        <v>2446.61</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8897,6 +9394,27 @@
       <c r="DR24" t="n">
         <v>10603.99</v>
       </c>
+      <c r="DS24" t="n">
+        <v>4466.24</v>
+      </c>
+      <c r="DT24" t="n">
+        <v>4548.23</v>
+      </c>
+      <c r="DU24" t="n">
+        <v>6574.41</v>
+      </c>
+      <c r="DV24" t="n">
+        <v>5766.309999999999</v>
+      </c>
+      <c r="DW24" t="n">
+        <v>5446.24</v>
+      </c>
+      <c r="DX24" t="n">
+        <v>7109.86</v>
+      </c>
+      <c r="DY24" t="n">
+        <v>3555.44</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9269,6 +9787,27 @@
       <c r="DR25" t="n">
         <v>12400.36</v>
       </c>
+      <c r="DS25" t="n">
+        <v>2992.34</v>
+      </c>
+      <c r="DT25" t="n">
+        <v>2824.69</v>
+      </c>
+      <c r="DU25" t="n">
+        <v>8660.450000000001</v>
+      </c>
+      <c r="DV25" t="n">
+        <v>2975.6</v>
+      </c>
+      <c r="DW25" t="n">
+        <v>4823.44</v>
+      </c>
+      <c r="DX25" t="n">
+        <v>14601.52</v>
+      </c>
+      <c r="DY25" t="n">
+        <v>2819.28</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9641,6 +10180,27 @@
       <c r="DR26" t="n">
         <v>3594.82</v>
       </c>
+      <c r="DS26" t="n">
+        <v>1583.87</v>
+      </c>
+      <c r="DT26" t="n">
+        <v>2020.86</v>
+      </c>
+      <c r="DU26" t="n">
+        <v>1740.22</v>
+      </c>
+      <c r="DV26" t="n">
+        <v>1429.08</v>
+      </c>
+      <c r="DW26" t="n">
+        <v>1686.36</v>
+      </c>
+      <c r="DX26" t="n">
+        <v>1765.1</v>
+      </c>
+      <c r="DY26" t="n">
+        <v>1007.1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -10013,6 +10573,27 @@
       <c r="DR27" t="n">
         <v>9958.400000000001</v>
       </c>
+      <c r="DS27" t="n">
+        <v>1594.05</v>
+      </c>
+      <c r="DT27" t="n">
+        <v>2704.93</v>
+      </c>
+      <c r="DU27" t="n">
+        <v>2809.92</v>
+      </c>
+      <c r="DV27" t="n">
+        <v>2204.76</v>
+      </c>
+      <c r="DW27" t="n">
+        <v>2856.12</v>
+      </c>
+      <c r="DX27" t="n">
+        <v>6147.46</v>
+      </c>
+      <c r="DY27" t="n">
+        <v>3723.94</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -10385,6 +10966,27 @@
       <c r="DR28" t="n">
         <v>18.8</v>
       </c>
+      <c r="DS28" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="DT28" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="DU28" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="DV28" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW28" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX28" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="DY28" t="n">
+        <v>43.6</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -10756,6 +11358,27 @@
       </c>
       <c r="DR29" t="n">
         <v>3.6</v>
+      </c>
+      <c r="DS29" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="DT29" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="DU29" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="DV29" t="n">
+        <v>2</v>
+      </c>
+      <c r="DW29" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="DX29" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="DY29" t="n">
+        <v>1.7</v>
       </c>
     </row>
     <row r="30">
@@ -11047,6 +11670,27 @@
       <c r="DR30" t="n">
         <v>744.5400000000001</v>
       </c>
+      <c r="DS30" t="n">
+        <v>663.61</v>
+      </c>
+      <c r="DT30" t="n">
+        <v>623.5700000000001</v>
+      </c>
+      <c r="DU30" t="n">
+        <v>400.39</v>
+      </c>
+      <c r="DV30" t="n">
+        <v>403.4</v>
+      </c>
+      <c r="DW30" t="n">
+        <v>435.75</v>
+      </c>
+      <c r="DX30" t="n">
+        <v>517.7</v>
+      </c>
+      <c r="DY30" t="n">
+        <v>379.9</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -11419,6 +12063,27 @@
       <c r="DR31" t="n">
         <v>15350.76</v>
       </c>
+      <c r="DS31" t="n">
+        <v>2386.42</v>
+      </c>
+      <c r="DT31" t="n">
+        <v>3163.3</v>
+      </c>
+      <c r="DU31" t="n">
+        <v>2715</v>
+      </c>
+      <c r="DV31" t="n">
+        <v>3245.04</v>
+      </c>
+      <c r="DW31" t="n">
+        <v>3464.3</v>
+      </c>
+      <c r="DX31" t="n">
+        <v>6448.97</v>
+      </c>
+      <c r="DY31" t="n">
+        <v>2419.61</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -11791,6 +12456,27 @@
       <c r="DR32" t="n">
         <v>9000.379999999999</v>
       </c>
+      <c r="DS32" t="n">
+        <v>2582.26</v>
+      </c>
+      <c r="DT32" t="n">
+        <v>3443.42</v>
+      </c>
+      <c r="DU32" t="n">
+        <v>4863.53</v>
+      </c>
+      <c r="DV32" t="n">
+        <v>3999.99</v>
+      </c>
+      <c r="DW32" t="n">
+        <v>4231.860000000001</v>
+      </c>
+      <c r="DX32" t="n">
+        <v>8235.66</v>
+      </c>
+      <c r="DY32" t="n">
+        <v>3753.95</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -12163,6 +12849,27 @@
       <c r="DR33" t="n">
         <v>6972.33</v>
       </c>
+      <c r="DS33" t="n">
+        <v>2251.02</v>
+      </c>
+      <c r="DT33" t="n">
+        <v>1655.31</v>
+      </c>
+      <c r="DU33" t="n">
+        <v>2404.24</v>
+      </c>
+      <c r="DV33" t="n">
+        <v>1792.75</v>
+      </c>
+      <c r="DW33" t="n">
+        <v>2202.71</v>
+      </c>
+      <c r="DX33" t="n">
+        <v>6945.26</v>
+      </c>
+      <c r="DY33" t="n">
+        <v>2125.57</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -12535,6 +13242,27 @@
       <c r="DR34" t="n">
         <v>2429.17</v>
       </c>
+      <c r="DS34" t="n">
+        <v>2922.22</v>
+      </c>
+      <c r="DT34" t="n">
+        <v>3988.12</v>
+      </c>
+      <c r="DU34" t="n">
+        <v>3137.83</v>
+      </c>
+      <c r="DV34" t="n">
+        <v>3184.39</v>
+      </c>
+      <c r="DW34" t="n">
+        <v>4128.53</v>
+      </c>
+      <c r="DX34" t="n">
+        <v>4248.12</v>
+      </c>
+      <c r="DY34" t="n">
+        <v>1555.87</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -12907,6 +13635,27 @@
       <c r="DR35" t="n">
         <v>2285.11</v>
       </c>
+      <c r="DS35" t="n">
+        <v>1341.74</v>
+      </c>
+      <c r="DT35" t="n">
+        <v>1075.34</v>
+      </c>
+      <c r="DU35" t="n">
+        <v>1109.61</v>
+      </c>
+      <c r="DV35" t="n">
+        <v>1429.88</v>
+      </c>
+      <c r="DW35" t="n">
+        <v>1463.98</v>
+      </c>
+      <c r="DX35" t="n">
+        <v>1578.15</v>
+      </c>
+      <c r="DY35" t="n">
+        <v>1481.05</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -13278,6 +14027,27 @@
       </c>
       <c r="DR36" t="n">
         <v>517.28</v>
+      </c>
+      <c r="DS36" t="n">
+        <v>99.24000000000001</v>
+      </c>
+      <c r="DT36" t="n">
+        <v>132.08</v>
+      </c>
+      <c r="DU36" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="DV36" t="n">
+        <v>279.48</v>
+      </c>
+      <c r="DW36" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="DX36" t="n">
+        <v>226</v>
+      </c>
+      <c r="DY36" t="n">
+        <v>98.66</v>
       </c>
     </row>
     <row r="37">
@@ -13473,6 +14243,27 @@
       <c r="DR37" t="n">
         <v>18068.25</v>
       </c>
+      <c r="DS37" t="n">
+        <v>1999.86</v>
+      </c>
+      <c r="DT37" t="n">
+        <v>2813.21</v>
+      </c>
+      <c r="DU37" t="n">
+        <v>3152.38</v>
+      </c>
+      <c r="DV37" t="n">
+        <v>2634.39</v>
+      </c>
+      <c r="DW37" t="n">
+        <v>2757.33</v>
+      </c>
+      <c r="DX37" t="n">
+        <v>6965.91</v>
+      </c>
+      <c r="DY37" t="n">
+        <v>2293.91</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -13667,6 +14458,27 @@
       <c r="DR38" t="n">
         <v>12413.16</v>
       </c>
+      <c r="DS38" t="n">
+        <v>2489.12</v>
+      </c>
+      <c r="DT38" t="n">
+        <v>1770.35</v>
+      </c>
+      <c r="DU38" t="n">
+        <v>7699.85</v>
+      </c>
+      <c r="DV38" t="n">
+        <v>2296.43</v>
+      </c>
+      <c r="DW38" t="n">
+        <v>2733.24</v>
+      </c>
+      <c r="DX38" t="n">
+        <v>9527.940000000001</v>
+      </c>
+      <c r="DY38" t="n">
+        <v>1344.41</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -13861,6 +14673,27 @@
       <c r="DR39" t="n">
         <v>1142.3</v>
       </c>
+      <c r="DS39" t="n">
+        <v>1319.15</v>
+      </c>
+      <c r="DT39" t="n">
+        <v>464.08</v>
+      </c>
+      <c r="DU39" t="n">
+        <v>401.05</v>
+      </c>
+      <c r="DV39" t="n">
+        <v>179.6</v>
+      </c>
+      <c r="DW39" t="n">
+        <v>443.45</v>
+      </c>
+      <c r="DX39" t="n">
+        <v>854.7</v>
+      </c>
+      <c r="DY39" t="n">
+        <v>103.1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -14233,6 +15066,27 @@
       <c r="DR40" t="n">
         <v>7538.52</v>
       </c>
+      <c r="DS40" t="n">
+        <v>2478.9</v>
+      </c>
+      <c r="DT40" t="n">
+        <v>2439.47</v>
+      </c>
+      <c r="DU40" t="n">
+        <v>2864.2</v>
+      </c>
+      <c r="DV40" t="n">
+        <v>2872.67</v>
+      </c>
+      <c r="DW40" t="n">
+        <v>2706.78</v>
+      </c>
+      <c r="DX40" t="n">
+        <v>4220.25</v>
+      </c>
+      <c r="DY40" t="n">
+        <v>4780.77</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -14605,6 +15459,27 @@
       <c r="DR41" t="n">
         <v>150420.46</v>
       </c>
+      <c r="DS41" t="n">
+        <v>47596.96</v>
+      </c>
+      <c r="DT41" t="n">
+        <v>47628.81</v>
+      </c>
+      <c r="DU41" t="n">
+        <v>63243.33</v>
+      </c>
+      <c r="DV41" t="n">
+        <v>46883.74</v>
+      </c>
+      <c r="DW41" t="n">
+        <v>52736.41</v>
+      </c>
+      <c r="DX41" t="n">
+        <v>94370.74000000001</v>
+      </c>
+      <c r="DY41" t="n">
+        <v>44838.53999999999</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -14976,6 +15851,27 @@
       </c>
       <c r="DR42" t="n">
         <v>3772.16</v>
+      </c>
+      <c r="DS42" t="n">
+        <v>4007.77</v>
+      </c>
+      <c r="DT42" t="n">
+        <v>2335.19</v>
+      </c>
+      <c r="DU42" t="n">
+        <v>2064.27</v>
+      </c>
+      <c r="DV42" t="n">
+        <v>1625.97</v>
+      </c>
+      <c r="DW42" t="n">
+        <v>1849.39</v>
+      </c>
+      <c r="DX42" t="n">
+        <v>1416.17</v>
+      </c>
+      <c r="DY42" t="n">
+        <v>2324.16</v>
       </c>
     </row>
     <row r="43">
@@ -15267,6 +16163,27 @@
       <c r="DR43" t="n">
         <v>29353.24</v>
       </c>
+      <c r="DS43" t="n">
+        <v>8467.16</v>
+      </c>
+      <c r="DT43" t="n">
+        <v>8032.34</v>
+      </c>
+      <c r="DU43" t="n">
+        <v>8225.02</v>
+      </c>
+      <c r="DV43" t="n">
+        <v>6628.299999999999</v>
+      </c>
+      <c r="DW43" t="n">
+        <v>7697.58</v>
+      </c>
+      <c r="DX43" t="n">
+        <v>9167.360000000001</v>
+      </c>
+      <c r="DY43" t="n">
+        <v>8580.290000000001</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -15639,6 +16556,27 @@
       <c r="DR44" t="n">
         <v>1876.09</v>
       </c>
+      <c r="DS44" t="n">
+        <v>1610.32</v>
+      </c>
+      <c r="DT44" t="n">
+        <v>1067</v>
+      </c>
+      <c r="DU44" t="n">
+        <v>1190.29</v>
+      </c>
+      <c r="DV44" t="n">
+        <v>936.8199999999999</v>
+      </c>
+      <c r="DW44" t="n">
+        <v>1068.99</v>
+      </c>
+      <c r="DX44" t="n">
+        <v>2008.72</v>
+      </c>
+      <c r="DY44" t="n">
+        <v>1050.06</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -16011,6 +16949,27 @@
       <c r="DR45" t="n">
         <v>4772.26</v>
       </c>
+      <c r="DS45" t="n">
+        <v>1632.1</v>
+      </c>
+      <c r="DT45" t="n">
+        <v>834.4499999999999</v>
+      </c>
+      <c r="DU45" t="n">
+        <v>1715.21</v>
+      </c>
+      <c r="DV45" t="n">
+        <v>1757.48</v>
+      </c>
+      <c r="DW45" t="n">
+        <v>1457.7</v>
+      </c>
+      <c r="DX45" t="n">
+        <v>2493.35</v>
+      </c>
+      <c r="DY45" t="n">
+        <v>1468.96</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -16383,6 +17342,27 @@
       <c r="DR46" t="n">
         <v>5168.280000000001</v>
       </c>
+      <c r="DS46" t="n">
+        <v>549.47</v>
+      </c>
+      <c r="DT46" t="n">
+        <v>727.1799999999999</v>
+      </c>
+      <c r="DU46" t="n">
+        <v>3248.83</v>
+      </c>
+      <c r="DV46" t="n">
+        <v>978.78</v>
+      </c>
+      <c r="DW46" t="n">
+        <v>787.7</v>
+      </c>
+      <c r="DX46" t="n">
+        <v>2309.5</v>
+      </c>
+      <c r="DY46" t="n">
+        <v>910.76</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -16755,6 +17735,27 @@
       <c r="DR47" t="n">
         <v>2715.72</v>
       </c>
+      <c r="DS47" t="n">
+        <v>555.2</v>
+      </c>
+      <c r="DT47" t="n">
+        <v>934.8</v>
+      </c>
+      <c r="DU47" t="n">
+        <v>877.25</v>
+      </c>
+      <c r="DV47" t="n">
+        <v>667.5</v>
+      </c>
+      <c r="DW47" t="n">
+        <v>1008.2</v>
+      </c>
+      <c r="DX47" t="n">
+        <v>720.25</v>
+      </c>
+      <c r="DY47" t="n">
+        <v>492.3000000000001</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -17127,6 +18128,27 @@
       <c r="DR48" t="n">
         <v>3235.58</v>
       </c>
+      <c r="DS48" t="n">
+        <v>694.36</v>
+      </c>
+      <c r="DT48" t="n">
+        <v>910.6300000000001</v>
+      </c>
+      <c r="DU48" t="n">
+        <v>592.5700000000001</v>
+      </c>
+      <c r="DV48" t="n">
+        <v>1041.58</v>
+      </c>
+      <c r="DW48" t="n">
+        <v>1239.36</v>
+      </c>
+      <c r="DX48" t="n">
+        <v>2347.63</v>
+      </c>
+      <c r="DY48" t="n">
+        <v>1570.65</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -17499,6 +18521,27 @@
       <c r="DR49" t="n">
         <v>0.4</v>
       </c>
+      <c r="DS49" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT49" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU49" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="DV49" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW49" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX49" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="DY49" t="n">
+        <v>2.2</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -17870,6 +18913,27 @@
       </c>
       <c r="DR50" t="n">
         <v>6.1</v>
+      </c>
+      <c r="DS50" t="n">
+        <v>5</v>
+      </c>
+      <c r="DT50" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="DU50" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="DV50" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="DW50" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="DX50" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="DY50" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="51">
@@ -18161,6 +19225,27 @@
       <c r="DR51" t="n">
         <v>78.62</v>
       </c>
+      <c r="DS51" t="n">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="DT51" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="DU51" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="DV51" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="DW51" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="DX51" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="DY51" t="n">
+        <v>49.2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -18533,6 +19618,27 @@
       <c r="DR52" t="n">
         <v>1029.92</v>
       </c>
+      <c r="DS52" t="n">
+        <v>1469.9</v>
+      </c>
+      <c r="DT52" t="n">
+        <v>903.7</v>
+      </c>
+      <c r="DU52" t="n">
+        <v>1540.2</v>
+      </c>
+      <c r="DV52" t="n">
+        <v>962.22</v>
+      </c>
+      <c r="DW52" t="n">
+        <v>1525.3</v>
+      </c>
+      <c r="DX52" t="n">
+        <v>2182.3</v>
+      </c>
+      <c r="DY52" t="n">
+        <v>646.8</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -18905,6 +20011,27 @@
       <c r="DR53" t="n">
         <v>3056.44</v>
       </c>
+      <c r="DS53" t="n">
+        <v>802.51</v>
+      </c>
+      <c r="DT53" t="n">
+        <v>900.05</v>
+      </c>
+      <c r="DU53" t="n">
+        <v>1034.46</v>
+      </c>
+      <c r="DV53" t="n">
+        <v>1049.59</v>
+      </c>
+      <c r="DW53" t="n">
+        <v>1000.72</v>
+      </c>
+      <c r="DX53" t="n">
+        <v>1661.76</v>
+      </c>
+      <c r="DY53" t="n">
+        <v>642.3200000000001</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -19277,6 +20404,27 @@
       <c r="DR54" t="n">
         <v>7053.880000000001</v>
       </c>
+      <c r="DS54" t="n">
+        <v>1336.21</v>
+      </c>
+      <c r="DT54" t="n">
+        <v>779.29</v>
+      </c>
+      <c r="DU54" t="n">
+        <v>1358.98</v>
+      </c>
+      <c r="DV54" t="n">
+        <v>1678.28</v>
+      </c>
+      <c r="DW54" t="n">
+        <v>1322.31</v>
+      </c>
+      <c r="DX54" t="n">
+        <v>3725.33</v>
+      </c>
+      <c r="DY54" t="n">
+        <v>873.8399999999999</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -19649,6 +20797,27 @@
       <c r="DR55" t="n">
         <v>723.39</v>
       </c>
+      <c r="DS55" t="n">
+        <v>391.11</v>
+      </c>
+      <c r="DT55" t="n">
+        <v>263.5</v>
+      </c>
+      <c r="DU55" t="n">
+        <v>366.41</v>
+      </c>
+      <c r="DV55" t="n">
+        <v>216.41</v>
+      </c>
+      <c r="DW55" t="n">
+        <v>1214.16</v>
+      </c>
+      <c r="DX55" t="n">
+        <v>1154.83</v>
+      </c>
+      <c r="DY55" t="n">
+        <v>250.09</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -20021,6 +21190,27 @@
       <c r="DR56" t="n">
         <v>1488.29</v>
       </c>
+      <c r="DS56" t="n">
+        <v>821.5</v>
+      </c>
+      <c r="DT56" t="n">
+        <v>819.0700000000001</v>
+      </c>
+      <c r="DU56" t="n">
+        <v>758.6600000000001</v>
+      </c>
+      <c r="DV56" t="n">
+        <v>872.49</v>
+      </c>
+      <c r="DW56" t="n">
+        <v>578.73</v>
+      </c>
+      <c r="DX56" t="n">
+        <v>1190.92</v>
+      </c>
+      <c r="DY56" t="n">
+        <v>1070.66</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -20392,6 +21582,27 @@
       </c>
       <c r="DR57" t="n">
         <v>603.6</v>
+      </c>
+      <c r="DS57" t="n">
+        <v>90.89999999999999</v>
+      </c>
+      <c r="DT57" t="n">
+        <v>123.95</v>
+      </c>
+      <c r="DU57" t="n">
+        <v>205.05</v>
+      </c>
+      <c r="DV57" t="n">
+        <v>131.6</v>
+      </c>
+      <c r="DW57" t="n">
+        <v>193.7</v>
+      </c>
+      <c r="DX57" t="n">
+        <v>305.8</v>
+      </c>
+      <c r="DY57" t="n">
+        <v>159.6</v>
       </c>
     </row>
     <row r="58">
@@ -20587,6 +21798,27 @@
       <c r="DR58" t="n">
         <v>6699.51</v>
       </c>
+      <c r="DS58" t="n">
+        <v>1165.51</v>
+      </c>
+      <c r="DT58" t="n">
+        <v>1732.91</v>
+      </c>
+      <c r="DU58" t="n">
+        <v>2347.51</v>
+      </c>
+      <c r="DV58" t="n">
+        <v>2583.73</v>
+      </c>
+      <c r="DW58" t="n">
+        <v>3180.08</v>
+      </c>
+      <c r="DX58" t="n">
+        <v>5805.7</v>
+      </c>
+      <c r="DY58" t="n">
+        <v>6077.3</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -20781,6 +22013,27 @@
       <c r="DR59" t="n">
         <v>2867.79</v>
       </c>
+      <c r="DS59" t="n">
+        <v>1237.31</v>
+      </c>
+      <c r="DT59" t="n">
+        <v>1032.43</v>
+      </c>
+      <c r="DU59" t="n">
+        <v>1470.26</v>
+      </c>
+      <c r="DV59" t="n">
+        <v>386.71</v>
+      </c>
+      <c r="DW59" t="n">
+        <v>372.01</v>
+      </c>
+      <c r="DX59" t="n">
+        <v>3180.35</v>
+      </c>
+      <c r="DY59" t="n">
+        <v>264.57</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -20975,6 +22228,27 @@
       <c r="DR60" t="n">
         <v>3939</v>
       </c>
+      <c r="DS60" t="n">
+        <v>2126</v>
+      </c>
+      <c r="DT60" t="n">
+        <v>413.5</v>
+      </c>
+      <c r="DU60" t="n">
+        <v>795.3000000000001</v>
+      </c>
+      <c r="DV60" t="n">
+        <v>373.6</v>
+      </c>
+      <c r="DW60" t="n">
+        <v>415.8</v>
+      </c>
+      <c r="DX60" t="n">
+        <v>1513.7</v>
+      </c>
+      <c r="DY60" t="n">
+        <v>751.7</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -21347,6 +22621,27 @@
       <c r="DR61" t="n">
         <v>4615.150000000001</v>
       </c>
+      <c r="DS61" t="n">
+        <v>1631.78</v>
+      </c>
+      <c r="DT61" t="n">
+        <v>1565.58</v>
+      </c>
+      <c r="DU61" t="n">
+        <v>1804.74</v>
+      </c>
+      <c r="DV61" t="n">
+        <v>1533.22</v>
+      </c>
+      <c r="DW61" t="n">
+        <v>1589.3</v>
+      </c>
+      <c r="DX61" t="n">
+        <v>3332.59</v>
+      </c>
+      <c r="DY61" t="n">
+        <v>2325.81</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -21719,6 +23014,27 @@
       <c r="DR62" t="n">
         <v>60187.38</v>
       </c>
+      <c r="DS62" t="n">
+        <v>19884.19</v>
+      </c>
+      <c r="DT62" t="n">
+        <v>16109.59</v>
+      </c>
+      <c r="DU62" t="n">
+        <v>22652.23</v>
+      </c>
+      <c r="DV62" t="n">
+        <v>18319.15</v>
+      </c>
+      <c r="DW62" t="n">
+        <v>19399.89</v>
+      </c>
+      <c r="DX62" t="n">
+        <v>37706.89</v>
+      </c>
+      <c r="DY62" t="n">
+        <v>22910.8</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -22090,6 +23406,27 @@
       </c>
       <c r="DR63" t="n">
         <v>1523.63</v>
+      </c>
+      <c r="DS63" t="n">
+        <v>1080.05</v>
+      </c>
+      <c r="DT63" t="n">
+        <v>307.15</v>
+      </c>
+      <c r="DU63" t="n">
+        <v>569.05</v>
+      </c>
+      <c r="DV63" t="n">
+        <v>522.74</v>
+      </c>
+      <c r="DW63" t="n">
+        <v>506.27</v>
+      </c>
+      <c r="DX63" t="n">
+        <v>1524.19</v>
+      </c>
+      <c r="DY63" t="n">
+        <v>2030.74</v>
       </c>
     </row>
     <row r="64">
@@ -22381,6 +23718,27 @@
       <c r="DR64" t="n">
         <v>8733.529999999999</v>
       </c>
+      <c r="DS64" t="n">
+        <v>2598.76</v>
+      </c>
+      <c r="DT64" t="n">
+        <v>2732.23</v>
+      </c>
+      <c r="DU64" t="n">
+        <v>2726.66</v>
+      </c>
+      <c r="DV64" t="n">
+        <v>2579.69</v>
+      </c>
+      <c r="DW64" t="n">
+        <v>1902.11</v>
+      </c>
+      <c r="DX64" t="n">
+        <v>2208.35</v>
+      </c>
+      <c r="DY64" t="n">
+        <v>2272.74</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -22753,6 +24111,27 @@
       <c r="DR65" t="n">
         <v>16241.4</v>
       </c>
+      <c r="DS65" t="n">
+        <v>11378.1</v>
+      </c>
+      <c r="DT65" t="n">
+        <v>12075.2</v>
+      </c>
+      <c r="DU65" t="n">
+        <v>18113.7</v>
+      </c>
+      <c r="DV65" t="n">
+        <v>20536.1</v>
+      </c>
+      <c r="DW65" t="n">
+        <v>24905.7</v>
+      </c>
+      <c r="DX65" t="n">
+        <v>28491.6</v>
+      </c>
+      <c r="DY65" t="n">
+        <v>25379.9</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -23125,6 +24504,27 @@
       <c r="DR66" t="n">
         <v>10873.8</v>
       </c>
+      <c r="DS66" t="n">
+        <v>3645.1</v>
+      </c>
+      <c r="DT66" t="n">
+        <v>7802.9</v>
+      </c>
+      <c r="DU66" t="n">
+        <v>14584.2</v>
+      </c>
+      <c r="DV66" t="n">
+        <v>12551</v>
+      </c>
+      <c r="DW66" t="n">
+        <v>15396.2</v>
+      </c>
+      <c r="DX66" t="n">
+        <v>26838.1</v>
+      </c>
+      <c r="DY66" t="n">
+        <v>22505.1</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -23497,6 +24897,27 @@
       <c r="DR67" t="n">
         <v>15652</v>
       </c>
+      <c r="DS67" t="n">
+        <v>18568.9</v>
+      </c>
+      <c r="DT67" t="n">
+        <v>16396.4</v>
+      </c>
+      <c r="DU67" t="n">
+        <v>20150.5</v>
+      </c>
+      <c r="DV67" t="n">
+        <v>19816.5</v>
+      </c>
+      <c r="DW67" t="n">
+        <v>23213</v>
+      </c>
+      <c r="DX67" t="n">
+        <v>33260.5</v>
+      </c>
+      <c r="DY67" t="n">
+        <v>31438.9</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -23869,6 +25290,27 @@
       <c r="DR68" t="n">
         <v>2702.3</v>
       </c>
+      <c r="DS68" t="n">
+        <v>1102.6</v>
+      </c>
+      <c r="DT68" t="n">
+        <v>1147.4</v>
+      </c>
+      <c r="DU68" t="n">
+        <v>1787.2</v>
+      </c>
+      <c r="DV68" t="n">
+        <v>2839.9</v>
+      </c>
+      <c r="DW68" t="n">
+        <v>5432.7</v>
+      </c>
+      <c r="DX68" t="n">
+        <v>4032.2</v>
+      </c>
+      <c r="DY68" t="n">
+        <v>2987.3</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -24241,6 +25683,27 @@
       <c r="DR69" t="n">
         <v>25435</v>
       </c>
+      <c r="DS69" t="n">
+        <v>11925.9</v>
+      </c>
+      <c r="DT69" t="n">
+        <v>13309</v>
+      </c>
+      <c r="DU69" t="n">
+        <v>17781.5</v>
+      </c>
+      <c r="DV69" t="n">
+        <v>21818.7</v>
+      </c>
+      <c r="DW69" t="n">
+        <v>24180</v>
+      </c>
+      <c r="DX69" t="n">
+        <v>30155.4</v>
+      </c>
+      <c r="DY69" t="n">
+        <v>28246.7</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -24613,6 +26076,27 @@
       <c r="DR70" t="n">
         <v>38.6</v>
       </c>
+      <c r="DS70" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="DT70" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="DU70" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="DV70" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="DW70" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="DX70" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="DY70" t="n">
+        <v>27.1</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -24984,6 +26468,27 @@
       </c>
       <c r="DR71" t="n">
         <v>0.2</v>
+      </c>
+      <c r="DS71" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="DT71" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="DU71" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="DV71" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="DW71" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="DX71" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="DY71" t="n">
+        <v>21.4</v>
       </c>
     </row>
     <row r="72">
@@ -25275,6 +26780,27 @@
       <c r="DR72" t="n">
         <v>5378.8</v>
       </c>
+      <c r="DS72" t="n">
+        <v>4112</v>
+      </c>
+      <c r="DT72" t="n">
+        <v>4463.5</v>
+      </c>
+      <c r="DU72" t="n">
+        <v>5183.200000000001</v>
+      </c>
+      <c r="DV72" t="n">
+        <v>6926.200000000001</v>
+      </c>
+      <c r="DW72" t="n">
+        <v>7755.3</v>
+      </c>
+      <c r="DX72" t="n">
+        <v>8152.1</v>
+      </c>
+      <c r="DY72" t="n">
+        <v>6931.2</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -25647,6 +27173,27 @@
       <c r="DR73" t="n">
         <v>18270.8</v>
       </c>
+      <c r="DS73" t="n">
+        <v>11870.5</v>
+      </c>
+      <c r="DT73" t="n">
+        <v>11950.3</v>
+      </c>
+      <c r="DU73" t="n">
+        <v>12804.8</v>
+      </c>
+      <c r="DV73" t="n">
+        <v>20325.3</v>
+      </c>
+      <c r="DW73" t="n">
+        <v>21966.6</v>
+      </c>
+      <c r="DX73" t="n">
+        <v>29428.1</v>
+      </c>
+      <c r="DY73" t="n">
+        <v>22638.4</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -26019,6 +27566,27 @@
       <c r="DR74" t="n">
         <v>9712.4</v>
       </c>
+      <c r="DS74" t="n">
+        <v>3211.2</v>
+      </c>
+      <c r="DT74" t="n">
+        <v>6609.1</v>
+      </c>
+      <c r="DU74" t="n">
+        <v>9067.299999999999</v>
+      </c>
+      <c r="DV74" t="n">
+        <v>19342.5</v>
+      </c>
+      <c r="DW74" t="n">
+        <v>35421.8</v>
+      </c>
+      <c r="DX74" t="n">
+        <v>40245.9</v>
+      </c>
+      <c r="DY74" t="n">
+        <v>28134.5</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -26391,6 +27959,27 @@
       <c r="DR75" t="n">
         <v>20918.7</v>
       </c>
+      <c r="DS75" t="n">
+        <v>4413.5</v>
+      </c>
+      <c r="DT75" t="n">
+        <v>7045.2</v>
+      </c>
+      <c r="DU75" t="n">
+        <v>16438.5</v>
+      </c>
+      <c r="DV75" t="n">
+        <v>16593.3</v>
+      </c>
+      <c r="DW75" t="n">
+        <v>25008.4</v>
+      </c>
+      <c r="DX75" t="n">
+        <v>33051.3</v>
+      </c>
+      <c r="DY75" t="n">
+        <v>22114.3</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -26763,6 +28352,27 @@
       <c r="DR76" t="n">
         <v>9839.799999999999</v>
       </c>
+      <c r="DS76" t="n">
+        <v>12296.7</v>
+      </c>
+      <c r="DT76" t="n">
+        <v>14608.5</v>
+      </c>
+      <c r="DU76" t="n">
+        <v>15571.1</v>
+      </c>
+      <c r="DV76" t="n">
+        <v>25665.2</v>
+      </c>
+      <c r="DW76" t="n">
+        <v>24862.8</v>
+      </c>
+      <c r="DX76" t="n">
+        <v>48355.4</v>
+      </c>
+      <c r="DY76" t="n">
+        <v>24434.4</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -27135,6 +28745,27 @@
       <c r="DR77" t="n">
         <v>5646.6</v>
       </c>
+      <c r="DS77" t="n">
+        <v>3000.2</v>
+      </c>
+      <c r="DT77" t="n">
+        <v>3036.2</v>
+      </c>
+      <c r="DU77" t="n">
+        <v>3195.7</v>
+      </c>
+      <c r="DV77" t="n">
+        <v>3601.1</v>
+      </c>
+      <c r="DW77" t="n">
+        <v>3887.4</v>
+      </c>
+      <c r="DX77" t="n">
+        <v>4754.3</v>
+      </c>
+      <c r="DY77" t="n">
+        <v>4682.9</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -27505,6 +29136,27 @@
         <v>0</v>
       </c>
       <c r="DR78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY78" t="n">
         <v>0</v>
       </c>
     </row>
@@ -27701,6 +29353,27 @@
       <c r="DR79" t="n">
         <v>16735.6</v>
       </c>
+      <c r="DS79" t="n">
+        <v>9509.799999999999</v>
+      </c>
+      <c r="DT79" t="n">
+        <v>12638.2</v>
+      </c>
+      <c r="DU79" t="n">
+        <v>20932.4</v>
+      </c>
+      <c r="DV79" t="n">
+        <v>26104.5</v>
+      </c>
+      <c r="DW79" t="n">
+        <v>30026.3</v>
+      </c>
+      <c r="DX79" t="n">
+        <v>43388.8</v>
+      </c>
+      <c r="DY79" t="n">
+        <v>37435.4</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -27895,6 +29568,27 @@
       <c r="DR80" t="n">
         <v>14631.7</v>
       </c>
+      <c r="DS80" t="n">
+        <v>10947.2</v>
+      </c>
+      <c r="DT80" t="n">
+        <v>9818</v>
+      </c>
+      <c r="DU80" t="n">
+        <v>16812.4</v>
+      </c>
+      <c r="DV80" t="n">
+        <v>19826.1</v>
+      </c>
+      <c r="DW80" t="n">
+        <v>19147.2</v>
+      </c>
+      <c r="DX80" t="n">
+        <v>27639</v>
+      </c>
+      <c r="DY80" t="n">
+        <v>21703.2</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -28089,6 +29783,27 @@
       <c r="DR81" t="n">
         <v>6779.9</v>
       </c>
+      <c r="DS81" t="n">
+        <v>943.5999999999999</v>
+      </c>
+      <c r="DT81" t="n">
+        <v>2536.8</v>
+      </c>
+      <c r="DU81" t="n">
+        <v>4311.9</v>
+      </c>
+      <c r="DV81" t="n">
+        <v>5524.8</v>
+      </c>
+      <c r="DW81" t="n">
+        <v>7606.299999999999</v>
+      </c>
+      <c r="DX81" t="n">
+        <v>5966.7</v>
+      </c>
+      <c r="DY81" t="n">
+        <v>10042.5</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -28461,6 +30176,27 @@
       <c r="DR82" t="n">
         <v>17260.2</v>
       </c>
+      <c r="DS82" t="n">
+        <v>15361.5</v>
+      </c>
+      <c r="DT82" t="n">
+        <v>15701.3</v>
+      </c>
+      <c r="DU82" t="n">
+        <v>19059</v>
+      </c>
+      <c r="DV82" t="n">
+        <v>21595.3</v>
+      </c>
+      <c r="DW82" t="n">
+        <v>23858.2</v>
+      </c>
+      <c r="DX82" t="n">
+        <v>29471.7</v>
+      </c>
+      <c r="DY82" t="n">
+        <v>28373.2</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -28833,6 +30569,27 @@
       <c r="DR83" t="n">
         <v>248141.8</v>
       </c>
+      <c r="DS83" t="n">
+        <v>173320.7</v>
+      </c>
+      <c r="DT83" t="n">
+        <v>193575</v>
+      </c>
+      <c r="DU83" t="n">
+        <v>262864.3</v>
+      </c>
+      <c r="DV83" t="n">
+        <v>327436.9</v>
+      </c>
+      <c r="DW83" t="n">
+        <v>390725.8</v>
+      </c>
+      <c r="DX83" t="n">
+        <v>500181.2</v>
+      </c>
+      <c r="DY83" t="n">
+        <v>407272.2</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -29204,6 +30961,27 @@
       </c>
       <c r="DR84" t="n">
         <v>23407.5</v>
+      </c>
+      <c r="DS84" t="n">
+        <v>17844.5</v>
+      </c>
+      <c r="DT84" t="n">
+        <v>18781.6</v>
+      </c>
+      <c r="DU84" t="n">
+        <v>22952.8</v>
+      </c>
+      <c r="DV84" t="n">
+        <v>34340.3</v>
+      </c>
+      <c r="DW84" t="n">
+        <v>38714.8</v>
+      </c>
+      <c r="DX84" t="n">
+        <v>45201.5</v>
+      </c>
+      <c r="DY84" t="n">
+        <v>46680.7</v>
       </c>
     </row>
     <row r="85">
@@ -29495,6 +31273,27 @@
       <c r="DR85" t="n">
         <v>28616.8</v>
       </c>
+      <c r="DS85" t="n">
+        <v>33158</v>
+      </c>
+      <c r="DT85" t="n">
+        <v>35623.7</v>
+      </c>
+      <c r="DU85" t="n">
+        <v>44086.4</v>
+      </c>
+      <c r="DV85" t="n">
+        <v>49990.5</v>
+      </c>
+      <c r="DW85" t="n">
+        <v>59303.1</v>
+      </c>
+      <c r="DX85" t="n">
+        <v>61702.9</v>
+      </c>
+      <c r="DY85" t="n">
+        <v>43495.5</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -29867,6 +31666,27 @@
       <c r="DR86" t="n">
         <v>717.2</v>
       </c>
+      <c r="DS86" t="n">
+        <v>606.5599999999999</v>
+      </c>
+      <c r="DT86" t="n">
+        <v>807.76</v>
+      </c>
+      <c r="DU86" t="n">
+        <v>799.6799999999999</v>
+      </c>
+      <c r="DV86" t="n">
+        <v>798.4</v>
+      </c>
+      <c r="DW86" t="n">
+        <v>819.9499999999999</v>
+      </c>
+      <c r="DX86" t="n">
+        <v>909.79</v>
+      </c>
+      <c r="DY86" t="n">
+        <v>525.54</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -30239,6 +32059,27 @@
       <c r="DR87" t="n">
         <v>3691.59</v>
       </c>
+      <c r="DS87" t="n">
+        <v>1267.28</v>
+      </c>
+      <c r="DT87" t="n">
+        <v>536.79</v>
+      </c>
+      <c r="DU87" t="n">
+        <v>2929.62</v>
+      </c>
+      <c r="DV87" t="n">
+        <v>1795.06</v>
+      </c>
+      <c r="DW87" t="n">
+        <v>1235.48</v>
+      </c>
+      <c r="DX87" t="n">
+        <v>2052.14</v>
+      </c>
+      <c r="DY87" t="n">
+        <v>1244.06</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -30611,6 +32452,27 @@
       <c r="DR88" t="n">
         <v>8213.899999999998</v>
       </c>
+      <c r="DS88" t="n">
+        <v>1113.56</v>
+      </c>
+      <c r="DT88" t="n">
+        <v>526.89</v>
+      </c>
+      <c r="DU88" t="n">
+        <v>3722.4</v>
+      </c>
+      <c r="DV88" t="n">
+        <v>775.3299999999999</v>
+      </c>
+      <c r="DW88" t="n">
+        <v>937.0599999999999</v>
+      </c>
+      <c r="DX88" t="n">
+        <v>3243.32</v>
+      </c>
+      <c r="DY88" t="n">
+        <v>950.9300000000001</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -30983,6 +32845,27 @@
       <c r="DR89" t="n">
         <v>1886.37</v>
       </c>
+      <c r="DS89" t="n">
+        <v>488.5500000000001</v>
+      </c>
+      <c r="DT89" t="n">
+        <v>574.5999999999999</v>
+      </c>
+      <c r="DU89" t="n">
+        <v>986.8299999999999</v>
+      </c>
+      <c r="DV89" t="n">
+        <v>812.85</v>
+      </c>
+      <c r="DW89" t="n">
+        <v>755.9300000000001</v>
+      </c>
+      <c r="DX89" t="n">
+        <v>2961.75</v>
+      </c>
+      <c r="DY89" t="n">
+        <v>744.45</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -31355,6 +33238,27 @@
       <c r="DR90" t="n">
         <v>3244.57</v>
       </c>
+      <c r="DS90" t="n">
+        <v>516.73</v>
+      </c>
+      <c r="DT90" t="n">
+        <v>716.8</v>
+      </c>
+      <c r="DU90" t="n">
+        <v>1048.98</v>
+      </c>
+      <c r="DV90" t="n">
+        <v>832.48</v>
+      </c>
+      <c r="DW90" t="n">
+        <v>946.63</v>
+      </c>
+      <c r="DX90" t="n">
+        <v>1415.91</v>
+      </c>
+      <c r="DY90" t="n">
+        <v>1527.06</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -31727,6 +33631,27 @@
       <c r="DR91" t="n">
         <v>0.8999999999999999</v>
       </c>
+      <c r="DS91" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="DT91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX91" t="n">
+        <v>5</v>
+      </c>
+      <c r="DY91" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -32098,6 +34023,27 @@
       </c>
       <c r="DR92" t="n">
         <v>1</v>
+      </c>
+      <c r="DS92" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="DT92" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="DU92" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="DV92" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="DW92" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="DX92" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="DY92" t="n">
+        <v>1.1</v>
       </c>
     </row>
     <row r="93">
@@ -32389,6 +34335,27 @@
       <c r="DR93" t="n">
         <v>212.13</v>
       </c>
+      <c r="DS93" t="n">
+        <v>108.39</v>
+      </c>
+      <c r="DT93" t="n">
+        <v>76.72</v>
+      </c>
+      <c r="DU93" t="n">
+        <v>63.56</v>
+      </c>
+      <c r="DV93" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="DW93" t="n">
+        <v>48</v>
+      </c>
+      <c r="DX93" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="DY93" t="n">
+        <v>128.01</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -32761,6 +34728,27 @@
       <c r="DR94" t="n">
         <v>4695.5</v>
       </c>
+      <c r="DS94" t="n">
+        <v>1880.47</v>
+      </c>
+      <c r="DT94" t="n">
+        <v>1806.25</v>
+      </c>
+      <c r="DU94" t="n">
+        <v>2109.5</v>
+      </c>
+      <c r="DV94" t="n">
+        <v>2102.1</v>
+      </c>
+      <c r="DW94" t="n">
+        <v>2455.4</v>
+      </c>
+      <c r="DX94" t="n">
+        <v>4804</v>
+      </c>
+      <c r="DY94" t="n">
+        <v>2430.85</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -33133,6 +35121,27 @@
       <c r="DR95" t="n">
         <v>3139.58</v>
       </c>
+      <c r="DS95" t="n">
+        <v>595.6700000000001</v>
+      </c>
+      <c r="DT95" t="n">
+        <v>629.36</v>
+      </c>
+      <c r="DU95" t="n">
+        <v>1093.13</v>
+      </c>
+      <c r="DV95" t="n">
+        <v>1348</v>
+      </c>
+      <c r="DW95" t="n">
+        <v>1610.72</v>
+      </c>
+      <c r="DX95" t="n">
+        <v>2238.47</v>
+      </c>
+      <c r="DY95" t="n">
+        <v>1548.44</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -33505,6 +35514,27 @@
       <c r="DR96" t="n">
         <v>2551.96</v>
       </c>
+      <c r="DS96" t="n">
+        <v>381</v>
+      </c>
+      <c r="DT96" t="n">
+        <v>375.04</v>
+      </c>
+      <c r="DU96" t="n">
+        <v>837.54</v>
+      </c>
+      <c r="DV96" t="n">
+        <v>357.73</v>
+      </c>
+      <c r="DW96" t="n">
+        <v>1127.95</v>
+      </c>
+      <c r="DX96" t="n">
+        <v>2110.63</v>
+      </c>
+      <c r="DY96" t="n">
+        <v>518.05</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -33877,6 +35907,27 @@
       <c r="DR97" t="n">
         <v>440.47</v>
       </c>
+      <c r="DS97" t="n">
+        <v>330.86</v>
+      </c>
+      <c r="DT97" t="n">
+        <v>141.87</v>
+      </c>
+      <c r="DU97" t="n">
+        <v>179.06</v>
+      </c>
+      <c r="DV97" t="n">
+        <v>1433.99</v>
+      </c>
+      <c r="DW97" t="n">
+        <v>149.31</v>
+      </c>
+      <c r="DX97" t="n">
+        <v>133.92</v>
+      </c>
+      <c r="DY97" t="n">
+        <v>153.09</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -34249,6 +36300,27 @@
       <c r="DR98" t="n">
         <v>544.1099999999999</v>
       </c>
+      <c r="DS98" t="n">
+        <v>533.78</v>
+      </c>
+      <c r="DT98" t="n">
+        <v>474.22</v>
+      </c>
+      <c r="DU98" t="n">
+        <v>443.29</v>
+      </c>
+      <c r="DV98" t="n">
+        <v>309.81</v>
+      </c>
+      <c r="DW98" t="n">
+        <v>628.26</v>
+      </c>
+      <c r="DX98" t="n">
+        <v>526.6799999999999</v>
+      </c>
+      <c r="DY98" t="n">
+        <v>250.73</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -34620,6 +36692,27 @@
       </c>
       <c r="DR99" t="n">
         <v>351.2</v>
+      </c>
+      <c r="DS99" t="n">
+        <v>151.54</v>
+      </c>
+      <c r="DT99" t="n">
+        <v>157.54</v>
+      </c>
+      <c r="DU99" t="n">
+        <v>131.34</v>
+      </c>
+      <c r="DV99" t="n">
+        <v>51.12</v>
+      </c>
+      <c r="DW99" t="n">
+        <v>132.39</v>
+      </c>
+      <c r="DX99" t="n">
+        <v>207.71</v>
+      </c>
+      <c r="DY99" t="n">
+        <v>176.88</v>
       </c>
     </row>
     <row r="100">
@@ -34815,6 +36908,27 @@
       <c r="DR100" t="n">
         <v>5726.09</v>
       </c>
+      <c r="DS100" t="n">
+        <v>612.23</v>
+      </c>
+      <c r="DT100" t="n">
+        <v>873.9499999999999</v>
+      </c>
+      <c r="DU100" t="n">
+        <v>1305.68</v>
+      </c>
+      <c r="DV100" t="n">
+        <v>1741.28</v>
+      </c>
+      <c r="DW100" t="n">
+        <v>2006.25</v>
+      </c>
+      <c r="DX100" t="n">
+        <v>4668.04</v>
+      </c>
+      <c r="DY100" t="n">
+        <v>1030.78</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -35009,6 +37123,27 @@
       <c r="DR101" t="n">
         <v>6680.27</v>
       </c>
+      <c r="DS101" t="n">
+        <v>689.58</v>
+      </c>
+      <c r="DT101" t="n">
+        <v>634.3099999999999</v>
+      </c>
+      <c r="DU101" t="n">
+        <v>3323.46</v>
+      </c>
+      <c r="DV101" t="n">
+        <v>811.6800000000001</v>
+      </c>
+      <c r="DW101" t="n">
+        <v>643.8</v>
+      </c>
+      <c r="DX101" t="n">
+        <v>4021.84</v>
+      </c>
+      <c r="DY101" t="n">
+        <v>801.7900000000001</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -35203,6 +37338,27 @@
       <c r="DR102" t="n">
         <v>441.06</v>
       </c>
+      <c r="DS102" t="n">
+        <v>338.6</v>
+      </c>
+      <c r="DT102" t="n">
+        <v>294.8</v>
+      </c>
+      <c r="DU102" t="n">
+        <v>306.9</v>
+      </c>
+      <c r="DV102" t="n">
+        <v>261.8</v>
+      </c>
+      <c r="DW102" t="n">
+        <v>699</v>
+      </c>
+      <c r="DX102" t="n">
+        <v>794.2</v>
+      </c>
+      <c r="DY102" t="n">
+        <v>246.9</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -35575,6 +37731,27 @@
       <c r="DR103" t="n">
         <v>1525.3</v>
       </c>
+      <c r="DS103" t="n">
+        <v>392.03</v>
+      </c>
+      <c r="DT103" t="n">
+        <v>423.63</v>
+      </c>
+      <c r="DU103" t="n">
+        <v>527.4400000000001</v>
+      </c>
+      <c r="DV103" t="n">
+        <v>904.24</v>
+      </c>
+      <c r="DW103" t="n">
+        <v>819.04</v>
+      </c>
+      <c r="DX103" t="n">
+        <v>1158.24</v>
+      </c>
+      <c r="DY103" t="n">
+        <v>573.3</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -35947,6 +38124,27 @@
       <c r="DR104" t="n">
         <v>53372.70999999999</v>
       </c>
+      <c r="DS104" t="n">
+        <v>14785.27</v>
+      </c>
+      <c r="DT104" t="n">
+        <v>13391.18</v>
+      </c>
+      <c r="DU104" t="n">
+        <v>24576.21</v>
+      </c>
+      <c r="DV104" t="n">
+        <v>18650.31</v>
+      </c>
+      <c r="DW104" t="n">
+        <v>19079.82</v>
+      </c>
+      <c r="DX104" t="n">
+        <v>35744.89</v>
+      </c>
+      <c r="DY104" t="n">
+        <v>16423.79</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -36318,6 +38516,27 @@
       </c>
       <c r="DR105" t="n">
         <v>443.65</v>
+      </c>
+      <c r="DS105" t="n">
+        <v>328.67</v>
+      </c>
+      <c r="DT105" t="n">
+        <v>73.45999999999999</v>
+      </c>
+      <c r="DU105" t="n">
+        <v>226.5</v>
+      </c>
+      <c r="DV105" t="n">
+        <v>324.2</v>
+      </c>
+      <c r="DW105" t="n">
+        <v>431.65</v>
+      </c>
+      <c r="DX105" t="n">
+        <v>492.27</v>
+      </c>
+      <c r="DY105" t="n">
+        <v>989.64</v>
       </c>
     </row>
     <row r="106">
@@ -36609,6 +38828,27 @@
       <c r="DR106" t="n">
         <v>8866.360000000001</v>
       </c>
+      <c r="DS106" t="n">
+        <v>4447.97</v>
+      </c>
+      <c r="DT106" t="n">
+        <v>4266.88</v>
+      </c>
+      <c r="DU106" t="n">
+        <v>4540.22</v>
+      </c>
+      <c r="DV106" t="n">
+        <v>3939.72</v>
+      </c>
+      <c r="DW106" t="n">
+        <v>3631.9</v>
+      </c>
+      <c r="DX106" t="n">
+        <v>3915</v>
+      </c>
+      <c r="DY106" t="n">
+        <v>2576.47</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -36981,6 +39221,27 @@
       <c r="DR107" t="n">
         <v>11438.74</v>
       </c>
+      <c r="DS107" t="n">
+        <v>8560.299999999999</v>
+      </c>
+      <c r="DT107" t="n">
+        <v>12551.51</v>
+      </c>
+      <c r="DU107" t="n">
+        <v>12385.3</v>
+      </c>
+      <c r="DV107" t="n">
+        <v>13015.9</v>
+      </c>
+      <c r="DW107" t="n">
+        <v>10609</v>
+      </c>
+      <c r="DX107" t="n">
+        <v>10408.6</v>
+      </c>
+      <c r="DY107" t="n">
+        <v>10639.7</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -37353,6 +39614,27 @@
       <c r="DR108" t="n">
         <v>254.2</v>
       </c>
+      <c r="DS108" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="DT108" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="DU108" t="n">
+        <v>18</v>
+      </c>
+      <c r="DV108" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="DW108" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="DX108" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="DY108" t="n">
+        <v>60.6</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -37725,6 +40007,27 @@
       <c r="DR109" t="n">
         <v>12207.96</v>
       </c>
+      <c r="DS109" t="n">
+        <v>12023.33</v>
+      </c>
+      <c r="DT109" t="n">
+        <v>10821.1</v>
+      </c>
+      <c r="DU109" t="n">
+        <v>12752.96</v>
+      </c>
+      <c r="DV109" t="n">
+        <v>13346.82</v>
+      </c>
+      <c r="DW109" t="n">
+        <v>11619.21</v>
+      </c>
+      <c r="DX109" t="n">
+        <v>10505.14</v>
+      </c>
+      <c r="DY109" t="n">
+        <v>10844.25</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -38097,6 +40400,27 @@
       <c r="DR110" t="n">
         <v>0.6</v>
       </c>
+      <c r="DS110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY110" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -38469,6 +40793,27 @@
       <c r="DR111" t="n">
         <v>5998.19</v>
       </c>
+      <c r="DS111" t="n">
+        <v>6376.96</v>
+      </c>
+      <c r="DT111" t="n">
+        <v>5574.809999999999</v>
+      </c>
+      <c r="DU111" t="n">
+        <v>6469.33</v>
+      </c>
+      <c r="DV111" t="n">
+        <v>6486.09</v>
+      </c>
+      <c r="DW111" t="n">
+        <v>6221.83</v>
+      </c>
+      <c r="DX111" t="n">
+        <v>6069.309999999999</v>
+      </c>
+      <c r="DY111" t="n">
+        <v>6186.68</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -38841,6 +41186,27 @@
       <c r="DR112" t="n">
         <v>0.1</v>
       </c>
+      <c r="DS112" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="DT112" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="DU112" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="DV112" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="DW112" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="DX112" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="DY112" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -39211,6 +41577,27 @@
         <v>0</v>
       </c>
       <c r="DR113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY113" t="n">
         <v>0</v>
       </c>
     </row>
@@ -39503,6 +41890,27 @@
       <c r="DR114" t="n">
         <v>29.7</v>
       </c>
+      <c r="DS114" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="DT114" t="n">
+        <v>5.300000000000001</v>
+      </c>
+      <c r="DU114" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="DV114" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="DW114" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="DX114" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="DY114" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -39875,6 +42283,27 @@
       <c r="DR115" t="n">
         <v>2167.03</v>
       </c>
+      <c r="DS115" t="n">
+        <v>1983.67</v>
+      </c>
+      <c r="DT115" t="n">
+        <v>1817.65</v>
+      </c>
+      <c r="DU115" t="n">
+        <v>2596.07</v>
+      </c>
+      <c r="DV115" t="n">
+        <v>1968.29</v>
+      </c>
+      <c r="DW115" t="n">
+        <v>1939.64</v>
+      </c>
+      <c r="DX115" t="n">
+        <v>1631.96</v>
+      </c>
+      <c r="DY115" t="n">
+        <v>1759.46</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -40247,6 +42676,27 @@
       <c r="DR116" t="n">
         <v>991.03</v>
       </c>
+      <c r="DS116" t="n">
+        <v>972.64</v>
+      </c>
+      <c r="DT116" t="n">
+        <v>1047.88</v>
+      </c>
+      <c r="DU116" t="n">
+        <v>1179.17</v>
+      </c>
+      <c r="DV116" t="n">
+        <v>989.24</v>
+      </c>
+      <c r="DW116" t="n">
+        <v>1101.94</v>
+      </c>
+      <c r="DX116" t="n">
+        <v>1008.55</v>
+      </c>
+      <c r="DY116" t="n">
+        <v>912.9300000000001</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -40619,6 +43069,27 @@
       <c r="DR117" t="n">
         <v>1132.22</v>
       </c>
+      <c r="DS117" t="n">
+        <v>1000.83</v>
+      </c>
+      <c r="DT117" t="n">
+        <v>892.11</v>
+      </c>
+      <c r="DU117" t="n">
+        <v>877.7400000000001</v>
+      </c>
+      <c r="DV117" t="n">
+        <v>1046.8</v>
+      </c>
+      <c r="DW117" t="n">
+        <v>920.1300000000001</v>
+      </c>
+      <c r="DX117" t="n">
+        <v>1090.89</v>
+      </c>
+      <c r="DY117" t="n">
+        <v>866.5699999999999</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -40991,6 +43462,27 @@
       <c r="DR118" t="n">
         <v>1539.94</v>
       </c>
+      <c r="DS118" t="n">
+        <v>1481.59</v>
+      </c>
+      <c r="DT118" t="n">
+        <v>1377.83</v>
+      </c>
+      <c r="DU118" t="n">
+        <v>1435.98</v>
+      </c>
+      <c r="DV118" t="n">
+        <v>1111.97</v>
+      </c>
+      <c r="DW118" t="n">
+        <v>1062.91</v>
+      </c>
+      <c r="DX118" t="n">
+        <v>988.78</v>
+      </c>
+      <c r="DY118" t="n">
+        <v>1083.18</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -41363,6 +43855,27 @@
       <c r="DR119" t="n">
         <v>41.06</v>
       </c>
+      <c r="DS119" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="DT119" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="DU119" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="DV119" t="n">
+        <v>5.600000000000001</v>
+      </c>
+      <c r="DW119" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="DX119" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="DY119" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -41734,6 +44247,27 @@
       </c>
       <c r="DR120" t="n">
         <v>754.21</v>
+      </c>
+      <c r="DS120" t="n">
+        <v>508.83</v>
+      </c>
+      <c r="DT120" t="n">
+        <v>427.6</v>
+      </c>
+      <c r="DU120" t="n">
+        <v>618.8</v>
+      </c>
+      <c r="DV120" t="n">
+        <v>1039.88</v>
+      </c>
+      <c r="DW120" t="n">
+        <v>730.33</v>
+      </c>
+      <c r="DX120" t="n">
+        <v>876.72</v>
+      </c>
+      <c r="DY120" t="n">
+        <v>911.41</v>
       </c>
     </row>
     <row r="121">
@@ -41929,6 +44463,27 @@
       <c r="DR121" t="n">
         <v>2226</v>
       </c>
+      <c r="DS121" t="n">
+        <v>1879.2</v>
+      </c>
+      <c r="DT121" t="n">
+        <v>1683.5</v>
+      </c>
+      <c r="DU121" t="n">
+        <v>1821.7</v>
+      </c>
+      <c r="DV121" t="n">
+        <v>2239.8</v>
+      </c>
+      <c r="DW121" t="n">
+        <v>2224.7</v>
+      </c>
+      <c r="DX121" t="n">
+        <v>1720.7</v>
+      </c>
+      <c r="DY121" t="n">
+        <v>2036.8</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -42123,6 +44678,27 @@
       <c r="DR122" t="n">
         <v>57.2</v>
       </c>
+      <c r="DS122" t="n">
+        <v>279.8</v>
+      </c>
+      <c r="DT122" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="DU122" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="DV122" t="n">
+        <v>124.4</v>
+      </c>
+      <c r="DW122" t="n">
+        <v>280.2</v>
+      </c>
+      <c r="DX122" t="n">
+        <v>175.8</v>
+      </c>
+      <c r="DY122" t="n">
+        <v>26.8</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -42317,6 +44893,27 @@
       <c r="DR123" t="n">
         <v>12.6</v>
       </c>
+      <c r="DS123" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT123" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU123" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV123" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW123" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX123" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY123" t="n">
+        <v>9.5</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -42689,6 +45286,27 @@
       <c r="DR124" t="n">
         <v>449.35</v>
       </c>
+      <c r="DS124" t="n">
+        <v>319.17</v>
+      </c>
+      <c r="DT124" t="n">
+        <v>252.85</v>
+      </c>
+      <c r="DU124" t="n">
+        <v>234.53</v>
+      </c>
+      <c r="DV124" t="n">
+        <v>559.95</v>
+      </c>
+      <c r="DW124" t="n">
+        <v>564.4299999999999</v>
+      </c>
+      <c r="DX124" t="n">
+        <v>819.9599999999999</v>
+      </c>
+      <c r="DY124" t="n">
+        <v>914.2800000000001</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -43061,6 +45679,27 @@
       <c r="DR125" t="n">
         <v>40228.95</v>
       </c>
+      <c r="DS125" t="n">
+        <v>36670.56999999999</v>
+      </c>
+      <c r="DT125" t="n">
+        <v>37636.06</v>
+      </c>
+      <c r="DU125" t="n">
+        <v>41911.52</v>
+      </c>
+      <c r="DV125" t="n">
+        <v>43312.81</v>
+      </c>
+      <c r="DW125" t="n">
+        <v>38741.79</v>
+      </c>
+      <c r="DX125" t="n">
+        <v>37016.73</v>
+      </c>
+      <c r="DY125" t="n">
+        <v>37862.91</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -43432,6 +46071,27 @@
       </c>
       <c r="DR126" t="n">
         <v>363.28</v>
+      </c>
+      <c r="DS126" t="n">
+        <v>414.0500000000001</v>
+      </c>
+      <c r="DT126" t="n">
+        <v>496.82</v>
+      </c>
+      <c r="DU126" t="n">
+        <v>705.66</v>
+      </c>
+      <c r="DV126" t="n">
+        <v>574.51</v>
+      </c>
+      <c r="DW126" t="n">
+        <v>682.0100000000001</v>
+      </c>
+      <c r="DX126" t="n">
+        <v>730.13</v>
+      </c>
+      <c r="DY126" t="n">
+        <v>978.5500000000001</v>
       </c>
     </row>
     <row r="127">
@@ -43723,6 +46383,27 @@
       <c r="DR127" t="n">
         <v>565.34</v>
       </c>
+      <c r="DS127" t="n">
+        <v>810.6</v>
+      </c>
+      <c r="DT127" t="n">
+        <v>641.64</v>
+      </c>
+      <c r="DU127" t="n">
+        <v>802.3000000000001</v>
+      </c>
+      <c r="DV127" t="n">
+        <v>750.0700000000001</v>
+      </c>
+      <c r="DW127" t="n">
+        <v>754.3099999999999</v>
+      </c>
+      <c r="DX127" t="n">
+        <v>925.6700000000001</v>
+      </c>
+      <c r="DY127" t="n">
+        <v>627.5999999999999</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -44095,6 +46776,27 @@
       <c r="DR128" t="n">
         <v>480.05</v>
       </c>
+      <c r="DS128" t="n">
+        <v>263.72</v>
+      </c>
+      <c r="DT128" t="n">
+        <v>340.79</v>
+      </c>
+      <c r="DU128" t="n">
+        <v>447.27</v>
+      </c>
+      <c r="DV128" t="n">
+        <v>467.44</v>
+      </c>
+      <c r="DW128" t="n">
+        <v>306.14</v>
+      </c>
+      <c r="DX128" t="n">
+        <v>694.22</v>
+      </c>
+      <c r="DY128" t="n">
+        <v>803.75</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -44467,6 +47169,27 @@
       <c r="DR129" t="n">
         <v>20.6</v>
       </c>
+      <c r="DS129" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="DT129" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="DU129" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="DV129" t="n">
+        <v>97.90000000000001</v>
+      </c>
+      <c r="DW129" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="DX129" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="DY129" t="n">
+        <v>41.1</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -44839,6 +47562,27 @@
       <c r="DR130" t="n">
         <v>156.2</v>
       </c>
+      <c r="DS130" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="DT130" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="DU130" t="n">
+        <v>170.6</v>
+      </c>
+      <c r="DV130" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="DW130" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="DX130" t="n">
+        <v>38</v>
+      </c>
+      <c r="DY130" t="n">
+        <v>26.9</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -45211,6 +47955,27 @@
       <c r="DR131" t="n">
         <v>0</v>
       </c>
+      <c r="DS131" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT131" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU131" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV131" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW131" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX131" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY131" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -45583,6 +48348,27 @@
       <c r="DR132" t="n">
         <v>513.21</v>
       </c>
+      <c r="DS132" t="n">
+        <v>347.69</v>
+      </c>
+      <c r="DT132" t="n">
+        <v>288.64</v>
+      </c>
+      <c r="DU132" t="n">
+        <v>272.95</v>
+      </c>
+      <c r="DV132" t="n">
+        <v>274.8100000000001</v>
+      </c>
+      <c r="DW132" t="n">
+        <v>287.1</v>
+      </c>
+      <c r="DX132" t="n">
+        <v>368.67</v>
+      </c>
+      <c r="DY132" t="n">
+        <v>268.94</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -45955,6 +48741,27 @@
       <c r="DR133" t="n">
         <v>0</v>
       </c>
+      <c r="DS133" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT133" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU133" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV133" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW133" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX133" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY133" t="n">
+        <v>2.2</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -46326,6 +49133,27 @@
       </c>
       <c r="DR134" t="n">
         <v>0.1</v>
+      </c>
+      <c r="DS134" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT134" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU134" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV134" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW134" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX134" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY134" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="135">
@@ -46617,6 +49445,27 @@
       <c r="DR135" t="n">
         <v>20.2</v>
       </c>
+      <c r="DS135" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="DT135" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="DU135" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="DV135" t="n">
+        <v>1</v>
+      </c>
+      <c r="DW135" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="DX135" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="DY135" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -46989,6 +49838,27 @@
       <c r="DR136" t="n">
         <v>26.9</v>
       </c>
+      <c r="DS136" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="DT136" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="DU136" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="DV136" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="DW136" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="DX136" t="n">
+        <v>83.19999999999999</v>
+      </c>
+      <c r="DY136" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -47361,6 +50231,27 @@
       <c r="DR137" t="n">
         <v>168.9</v>
       </c>
+      <c r="DS137" t="n">
+        <v>136.6</v>
+      </c>
+      <c r="DT137" t="n">
+        <v>168.6</v>
+      </c>
+      <c r="DU137" t="n">
+        <v>232.8</v>
+      </c>
+      <c r="DV137" t="n">
+        <v>213.8</v>
+      </c>
+      <c r="DW137" t="n">
+        <v>223.4</v>
+      </c>
+      <c r="DX137" t="n">
+        <v>180.1</v>
+      </c>
+      <c r="DY137" t="n">
+        <v>166.6</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -47733,6 +50624,27 @@
       <c r="DR138" t="n">
         <v>934.6600000000001</v>
       </c>
+      <c r="DS138" t="n">
+        <v>614.67</v>
+      </c>
+      <c r="DT138" t="n">
+        <v>650.0400000000001</v>
+      </c>
+      <c r="DU138" t="n">
+        <v>879.3000000000001</v>
+      </c>
+      <c r="DV138" t="n">
+        <v>1052.23</v>
+      </c>
+      <c r="DW138" t="n">
+        <v>1181.78</v>
+      </c>
+      <c r="DX138" t="n">
+        <v>1087.37</v>
+      </c>
+      <c r="DY138" t="n">
+        <v>842.5799999999999</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -48105,6 +51017,27 @@
       <c r="DR139" t="n">
         <v>528.1900000000001</v>
       </c>
+      <c r="DS139" t="n">
+        <v>829.5600000000001</v>
+      </c>
+      <c r="DT139" t="n">
+        <v>555.74</v>
+      </c>
+      <c r="DU139" t="n">
+        <v>195.42</v>
+      </c>
+      <c r="DV139" t="n">
+        <v>85.87</v>
+      </c>
+      <c r="DW139" t="n">
+        <v>116.23</v>
+      </c>
+      <c r="DX139" t="n">
+        <v>195.09</v>
+      </c>
+      <c r="DY139" t="n">
+        <v>183.42</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -48477,6 +51410,27 @@
       <c r="DR140" t="n">
         <v>5.2</v>
       </c>
+      <c r="DS140" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="DT140" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="DU140" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="DV140" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="DW140" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="DX140" t="n">
+        <v>3</v>
+      </c>
+      <c r="DY140" t="n">
+        <v>3.2</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -48847,6 +51801,27 @@
         <v>0</v>
       </c>
       <c r="DR141" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS141" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT141" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU141" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV141" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW141" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX141" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY141" t="n">
         <v>0</v>
       </c>
     </row>
@@ -49043,6 +52018,27 @@
       <c r="DR142" t="n">
         <v>152.1</v>
       </c>
+      <c r="DS142" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="DT142" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="DU142" t="n">
+        <v>94.90000000000001</v>
+      </c>
+      <c r="DV142" t="n">
+        <v>112.6</v>
+      </c>
+      <c r="DW142" t="n">
+        <v>147.4</v>
+      </c>
+      <c r="DX142" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="DY142" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -49237,6 +52233,27 @@
       <c r="DR143" t="n">
         <v>175.4</v>
       </c>
+      <c r="DS143" t="n">
+        <v>130.43</v>
+      </c>
+      <c r="DT143" t="n">
+        <v>138.3</v>
+      </c>
+      <c r="DU143" t="n">
+        <v>208.34</v>
+      </c>
+      <c r="DV143" t="n">
+        <v>165.61</v>
+      </c>
+      <c r="DW143" t="n">
+        <v>174.63</v>
+      </c>
+      <c r="DX143" t="n">
+        <v>590.36</v>
+      </c>
+      <c r="DY143" t="n">
+        <v>195.49</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -49431,6 +52448,27 @@
       <c r="DR144" t="n">
         <v>3.6</v>
       </c>
+      <c r="DS144" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="DT144" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="DU144" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="DV144" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW144" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="DX144" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="DY144" t="n">
+        <v>2.6</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -49803,6 +52841,27 @@
       <c r="DR145" t="n">
         <v>1662.16</v>
       </c>
+      <c r="DS145" t="n">
+        <v>1227.05</v>
+      </c>
+      <c r="DT145" t="n">
+        <v>1408.94</v>
+      </c>
+      <c r="DU145" t="n">
+        <v>1867.97</v>
+      </c>
+      <c r="DV145" t="n">
+        <v>1494.22</v>
+      </c>
+      <c r="DW145" t="n">
+        <v>1512.88</v>
+      </c>
+      <c r="DX145" t="n">
+        <v>1586.88</v>
+      </c>
+      <c r="DY145" t="n">
+        <v>1529.18</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -50175,6 +53234,27 @@
       <c r="DR146" t="n">
         <v>6873.080000000001</v>
       </c>
+      <c r="DS146" t="n">
+        <v>5485.690000000001</v>
+      </c>
+      <c r="DT146" t="n">
+        <v>5614.280000000001</v>
+      </c>
+      <c r="DU146" t="n">
+        <v>6217.26</v>
+      </c>
+      <c r="DV146" t="n">
+        <v>5888.23</v>
+      </c>
+      <c r="DW146" t="n">
+        <v>5581.13</v>
+      </c>
+      <c r="DX146" t="n">
+        <v>6429.809999999999</v>
+      </c>
+      <c r="DY146" t="n">
+        <v>6876.52</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -50546,6 +53626,27 @@
       </c>
       <c r="DR147" t="n">
         <v>2020.1</v>
+      </c>
+      <c r="DS147" t="n">
+        <v>1689.17</v>
+      </c>
+      <c r="DT147" t="n">
+        <v>1721.94</v>
+      </c>
+      <c r="DU147" t="n">
+        <v>1684</v>
+      </c>
+      <c r="DV147" t="n">
+        <v>1852.75</v>
+      </c>
+      <c r="DW147" t="n">
+        <v>1591.07</v>
+      </c>
+      <c r="DX147" t="n">
+        <v>1441.53</v>
+      </c>
+      <c r="DY147" t="n">
+        <v>2780.05</v>
       </c>
     </row>
     <row r="148">
@@ -50837,6 +53938,27 @@
       <c r="DR148" t="n">
         <v>5.7</v>
       </c>
+      <c r="DS148" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="DT148" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="DU148" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="DV148" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="DW148" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="DX148" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="DY148" t="n">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -51209,6 +54331,27 @@
       <c r="DR149" t="n">
         <v>55640.3</v>
       </c>
+      <c r="DS149" t="n">
+        <v>54329</v>
+      </c>
+      <c r="DT149" t="n">
+        <v>45131.6</v>
+      </c>
+      <c r="DU149" t="n">
+        <v>60384.8</v>
+      </c>
+      <c r="DV149" t="n">
+        <v>53061.5</v>
+      </c>
+      <c r="DW149" t="n">
+        <v>62239.8</v>
+      </c>
+      <c r="DX149" t="n">
+        <v>61806.39999999999</v>
+      </c>
+      <c r="DY149" t="n">
+        <v>62214.8</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -51581,6 +54724,27 @@
       <c r="DR150" t="n">
         <v>18775.5</v>
       </c>
+      <c r="DS150" t="n">
+        <v>20148.6</v>
+      </c>
+      <c r="DT150" t="n">
+        <v>17195.1</v>
+      </c>
+      <c r="DU150" t="n">
+        <v>19281.6</v>
+      </c>
+      <c r="DV150" t="n">
+        <v>19471.9</v>
+      </c>
+      <c r="DW150" t="n">
+        <v>19921.5</v>
+      </c>
+      <c r="DX150" t="n">
+        <v>19866.6</v>
+      </c>
+      <c r="DY150" t="n">
+        <v>21013.7</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -51953,6 +55117,27 @@
       <c r="DR151" t="n">
         <v>47398.59999999999</v>
       </c>
+      <c r="DS151" t="n">
+        <v>41510.5</v>
+      </c>
+      <c r="DT151" t="n">
+        <v>38920.1</v>
+      </c>
+      <c r="DU151" t="n">
+        <v>41024.7</v>
+      </c>
+      <c r="DV151" t="n">
+        <v>40330.8</v>
+      </c>
+      <c r="DW151" t="n">
+        <v>42775.49999999999</v>
+      </c>
+      <c r="DX151" t="n">
+        <v>38080.09999999999</v>
+      </c>
+      <c r="DY151" t="n">
+        <v>34238.1</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -52325,6 +55510,27 @@
       <c r="DR152" t="n">
         <v>3581.1</v>
       </c>
+      <c r="DS152" t="n">
+        <v>4789.5</v>
+      </c>
+      <c r="DT152" t="n">
+        <v>4333.4</v>
+      </c>
+      <c r="DU152" t="n">
+        <v>4701.3</v>
+      </c>
+      <c r="DV152" t="n">
+        <v>4444.1</v>
+      </c>
+      <c r="DW152" t="n">
+        <v>4447.7</v>
+      </c>
+      <c r="DX152" t="n">
+        <v>4083.3</v>
+      </c>
+      <c r="DY152" t="n">
+        <v>3883.1</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -52697,6 +55903,27 @@
       <c r="DR153" t="n">
         <v>4553.099999999999</v>
       </c>
+      <c r="DS153" t="n">
+        <v>2154.3</v>
+      </c>
+      <c r="DT153" t="n">
+        <v>2920.8</v>
+      </c>
+      <c r="DU153" t="n">
+        <v>3721</v>
+      </c>
+      <c r="DV153" t="n">
+        <v>4525.3</v>
+      </c>
+      <c r="DW153" t="n">
+        <v>6128.1</v>
+      </c>
+      <c r="DX153" t="n">
+        <v>6290.9</v>
+      </c>
+      <c r="DY153" t="n">
+        <v>6076.400000000001</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -53069,6 +56296,27 @@
       <c r="DR154" t="n">
         <v>15.1</v>
       </c>
+      <c r="DS154" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="DT154" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="DU154" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="DV154" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="DW154" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="DX154" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="DY154" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -53440,6 +56688,27 @@
       </c>
       <c r="DR155" t="n">
         <v>0.1</v>
+      </c>
+      <c r="DS155" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="DT155" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="DU155" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="DV155" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="DW155" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="DX155" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="DY155" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="156">
@@ -53731,6 +57000,27 @@
       <c r="DR156" t="n">
         <v>17266.1</v>
       </c>
+      <c r="DS156" t="n">
+        <v>15993</v>
+      </c>
+      <c r="DT156" t="n">
+        <v>15508.6</v>
+      </c>
+      <c r="DU156" t="n">
+        <v>19010</v>
+      </c>
+      <c r="DV156" t="n">
+        <v>18345.7</v>
+      </c>
+      <c r="DW156" t="n">
+        <v>20423.9</v>
+      </c>
+      <c r="DX156" t="n">
+        <v>20916.3</v>
+      </c>
+      <c r="DY156" t="n">
+        <v>21832</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -54103,6 +57393,27 @@
       <c r="DR157" t="n">
         <v>7000.5</v>
       </c>
+      <c r="DS157" t="n">
+        <v>4617.9</v>
+      </c>
+      <c r="DT157" t="n">
+        <v>4184.4</v>
+      </c>
+      <c r="DU157" t="n">
+        <v>6278</v>
+      </c>
+      <c r="DV157" t="n">
+        <v>6696</v>
+      </c>
+      <c r="DW157" t="n">
+        <v>6999.2</v>
+      </c>
+      <c r="DX157" t="n">
+        <v>10690.5</v>
+      </c>
+      <c r="DY157" t="n">
+        <v>13810</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -54475,6 +57786,27 @@
       <c r="DR158" t="n">
         <v>10530</v>
       </c>
+      <c r="DS158" t="n">
+        <v>8763.4</v>
+      </c>
+      <c r="DT158" t="n">
+        <v>10359.5</v>
+      </c>
+      <c r="DU158" t="n">
+        <v>10459.2</v>
+      </c>
+      <c r="DV158" t="n">
+        <v>11136.5</v>
+      </c>
+      <c r="DW158" t="n">
+        <v>10509</v>
+      </c>
+      <c r="DX158" t="n">
+        <v>13037.6</v>
+      </c>
+      <c r="DY158" t="n">
+        <v>11245.8</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -54847,6 +58179,27 @@
       <c r="DR159" t="n">
         <v>51088.60000000001</v>
       </c>
+      <c r="DS159" t="n">
+        <v>50601.1</v>
+      </c>
+      <c r="DT159" t="n">
+        <v>41905.6</v>
+      </c>
+      <c r="DU159" t="n">
+        <v>46816.9</v>
+      </c>
+      <c r="DV159" t="n">
+        <v>54373.40000000001</v>
+      </c>
+      <c r="DW159" t="n">
+        <v>54243.7</v>
+      </c>
+      <c r="DX159" t="n">
+        <v>56042.2</v>
+      </c>
+      <c r="DY159" t="n">
+        <v>54984.8</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -55219,6 +58572,27 @@
       <c r="DR160" t="n">
         <v>31412.9</v>
       </c>
+      <c r="DS160" t="n">
+        <v>33270.7</v>
+      </c>
+      <c r="DT160" t="n">
+        <v>25198</v>
+      </c>
+      <c r="DU160" t="n">
+        <v>28343.3</v>
+      </c>
+      <c r="DV160" t="n">
+        <v>34878.5</v>
+      </c>
+      <c r="DW160" t="n">
+        <v>35445.3</v>
+      </c>
+      <c r="DX160" t="n">
+        <v>33353.5</v>
+      </c>
+      <c r="DY160" t="n">
+        <v>32197.3</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -55591,6 +58965,27 @@
       <c r="DR161" t="n">
         <v>695.8</v>
       </c>
+      <c r="DS161" t="n">
+        <v>259</v>
+      </c>
+      <c r="DT161" t="n">
+        <v>356.7</v>
+      </c>
+      <c r="DU161" t="n">
+        <v>427.2</v>
+      </c>
+      <c r="DV161" t="n">
+        <v>681.7</v>
+      </c>
+      <c r="DW161" t="n">
+        <v>737.5</v>
+      </c>
+      <c r="DX161" t="n">
+        <v>837.8000000000001</v>
+      </c>
+      <c r="DY161" t="n">
+        <v>808.9</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -55962,6 +59357,27 @@
       </c>
       <c r="DR162" t="n">
         <v>41.1</v>
+      </c>
+      <c r="DS162" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="DT162" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="DU162" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="DV162" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="DW162" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="DX162" t="n">
+        <v>88</v>
+      </c>
+      <c r="DY162" t="n">
+        <v>87.8</v>
       </c>
     </row>
     <row r="163">
@@ -56157,6 +59573,27 @@
       <c r="DR163" t="n">
         <v>3916.9</v>
       </c>
+      <c r="DS163" t="n">
+        <v>2149</v>
+      </c>
+      <c r="DT163" t="n">
+        <v>3322.2</v>
+      </c>
+      <c r="DU163" t="n">
+        <v>4423.2</v>
+      </c>
+      <c r="DV163" t="n">
+        <v>5159.2</v>
+      </c>
+      <c r="DW163" t="n">
+        <v>5802.4</v>
+      </c>
+      <c r="DX163" t="n">
+        <v>6556.6</v>
+      </c>
+      <c r="DY163" t="n">
+        <v>7458.2</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -56351,6 +59788,27 @@
       <c r="DR164" t="n">
         <v>27657</v>
       </c>
+      <c r="DS164" t="n">
+        <v>25193.8</v>
+      </c>
+      <c r="DT164" t="n">
+        <v>28661.9</v>
+      </c>
+      <c r="DU164" t="n">
+        <v>27089.7</v>
+      </c>
+      <c r="DV164" t="n">
+        <v>29787.1</v>
+      </c>
+      <c r="DW164" t="n">
+        <v>27042.1</v>
+      </c>
+      <c r="DX164" t="n">
+        <v>28008.8</v>
+      </c>
+      <c r="DY164" t="n">
+        <v>27987.2</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -56545,6 +60003,27 @@
       <c r="DR165" t="n">
         <v>1780.6</v>
       </c>
+      <c r="DS165" t="n">
+        <v>1621.8</v>
+      </c>
+      <c r="DT165" t="n">
+        <v>1907.1</v>
+      </c>
+      <c r="DU165" t="n">
+        <v>2712.3</v>
+      </c>
+      <c r="DV165" t="n">
+        <v>2117.5</v>
+      </c>
+      <c r="DW165" t="n">
+        <v>2241.9</v>
+      </c>
+      <c r="DX165" t="n">
+        <v>4710.8</v>
+      </c>
+      <c r="DY165" t="n">
+        <v>2247.1</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -56917,6 +60396,27 @@
       <c r="DR166" t="n">
         <v>14834.9</v>
       </c>
+      <c r="DS166" t="n">
+        <v>15255.1</v>
+      </c>
+      <c r="DT166" t="n">
+        <v>13505.1</v>
+      </c>
+      <c r="DU166" t="n">
+        <v>14773.7</v>
+      </c>
+      <c r="DV166" t="n">
+        <v>16632.7</v>
+      </c>
+      <c r="DW166" t="n">
+        <v>16201</v>
+      </c>
+      <c r="DX166" t="n">
+        <v>16699.6</v>
+      </c>
+      <c r="DY166" t="n">
+        <v>18734.2</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -57289,6 +60789,27 @@
       <c r="DR167" t="n">
         <v>364206.5000000001</v>
       </c>
+      <c r="DS167" t="n">
+        <v>346859.4</v>
+      </c>
+      <c r="DT167" t="n">
+        <v>314262.0000000001</v>
+      </c>
+      <c r="DU167" t="n">
+        <v>359845</v>
+      </c>
+      <c r="DV167" t="n">
+        <v>378274.8</v>
+      </c>
+      <c r="DW167" t="n">
+        <v>397807.5</v>
+      </c>
+      <c r="DX167" t="n">
+        <v>407717.2999999999</v>
+      </c>
+      <c r="DY167" t="n">
+        <v>405302.8</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -57660,6 +61181,27 @@
       </c>
       <c r="DR168" t="n">
         <v>48441.5</v>
+      </c>
+      <c r="DS168" t="n">
+        <v>47327</v>
+      </c>
+      <c r="DT168" t="n">
+        <v>44265.4</v>
+      </c>
+      <c r="DU168" t="n">
+        <v>49073</v>
+      </c>
+      <c r="DV168" t="n">
+        <v>52808.8</v>
+      </c>
+      <c r="DW168" t="n">
+        <v>57261.1</v>
+      </c>
+      <c r="DX168" t="n">
+        <v>59281.5</v>
+      </c>
+      <c r="DY168" t="n">
+        <v>63008.60000000001</v>
       </c>
     </row>
     <row r="169">
@@ -57951,6 +61493,27 @@
       <c r="DR169" t="n">
         <v>19576.8</v>
       </c>
+      <c r="DS169" t="n">
+        <v>18830.5</v>
+      </c>
+      <c r="DT169" t="n">
+        <v>16545.6</v>
+      </c>
+      <c r="DU169" t="n">
+        <v>21272.4</v>
+      </c>
+      <c r="DV169" t="n">
+        <v>23757.1</v>
+      </c>
+      <c r="DW169" t="n">
+        <v>25319.1</v>
+      </c>
+      <c r="DX169" t="n">
+        <v>27352.3</v>
+      </c>
+      <c r="DY169" t="n">
+        <v>23460.7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>